<commit_message>
Atualiza resultados automáticos via CSV
</commit_message>
<xml_diff>
--- a/output/catalogo_csv_completo.xlsx
+++ b/output/catalogo_csv_completo.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Links API" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Links" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K163"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -430,7 +430,7 @@
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="45" customWidth="1" min="9" max="9"/>
     <col width="90" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -441,7 +441,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>anime_slug_used</t>
+          <t>query_used</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -496,22 +496,37 @@
           <t>Naruto</t>
         </is>
       </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Naruto</t>
+        </is>
+      </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Naruto Shippuden</t>
+          <t>Naruto</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -522,14 +537,19 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Boruto</t>
+          <t>Naruto Shippuden</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Naruto Shippuden</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -538,16 +558,26 @@
       <c r="D4" t="n">
         <v>1</v>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>One Piece</t>
+          <t>Naruto Shippuden</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -558,14 +588,19 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dragon Ball Z</t>
+          <t>Boruto</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Boruto</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -574,16 +609,26 @@
       <c r="D6" t="n">
         <v>1</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Dragon Ball Super</t>
+          <t>Boruto</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -594,14 +639,19 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Attack on Titan</t>
+          <t>One Piece</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>One Piece</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -610,16 +660,26 @@
       <c r="D8" t="n">
         <v>1</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Shingeki no Kyojin</t>
+          <t>One Piece</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -630,14 +690,19 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Demon Slayer</t>
+          <t>Dragon Ball Z</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dragon Ball Z</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -646,16 +711,26 @@
       <c r="D10" t="n">
         <v>1</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kimetsu no Yaiba</t>
+          <t>Dragon Ball Z</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -666,14 +741,19 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jujutsu Kaisen</t>
+          <t>Dragon Ball Super</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Dragon Ball Super</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -682,16 +762,26 @@
       <c r="D12" t="n">
         <v>1</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Death Note</t>
+          <t>Dragon Ball Super</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -702,14 +792,19 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Fullmetal Alchemist Brotherhood</t>
+          <t>Attack on Titan</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Attack on Titan</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -718,16 +813,26 @@
       <c r="D14" t="n">
         <v>1</v>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tokyo Ghoul</t>
+          <t>Attack on Titan</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -738,14 +843,19 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bleach</t>
+          <t>Shingeki no Kyojin</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Shingeki no Kyojin</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -754,16 +864,26 @@
       <c r="D16" t="n">
         <v>1</v>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bleach Thousand-Year Blood War</t>
+          <t>Shingeki no Kyojin</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -774,14 +894,19 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Hunter x Hunter</t>
+          <t>Demon Slayer</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Demon Slayer</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -790,16 +915,26 @@
       <c r="D18" t="n">
         <v>1</v>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Black Clover</t>
+          <t>Demon Slayer</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -810,14 +945,19 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>My Hero Academia</t>
+          <t>Kimetsu no Yaiba</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Kimetsu no Yaiba</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -826,16 +966,26 @@
       <c r="D20" t="n">
         <v>1</v>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Boku no Hero Academia</t>
+          <t>Kimetsu no Yaiba</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -846,14 +996,19 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Chainsaw Man</t>
+          <t>Jujutsu Kaisen</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Jujutsu Kaisen</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -862,16 +1017,26 @@
       <c r="D22" t="n">
         <v>1</v>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Solo Leveling</t>
+          <t>Jujutsu Kaisen</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -882,14 +1047,19 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Sword Art Online</t>
+          <t>Death Note</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Death Note</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -898,16 +1068,26 @@
       <c r="D24" t="n">
         <v>1</v>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Fairy Tail</t>
+          <t>Death Note</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -918,14 +1098,19 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Blue Lock</t>
+          <t>Fullmetal Alchemist Brotherhood</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Fullmetal Alchemist Brotherhood</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -934,16 +1119,26 @@
       <c r="D26" t="n">
         <v>1</v>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Haikyuu</t>
+          <t>Fullmetal Alchemist Brotherhood</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -954,14 +1149,19 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Kuroko no Basket</t>
+          <t>Tokyo Ghoul</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Tokyo Ghoul</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -970,16 +1170,26 @@
       <c r="D28" t="n">
         <v>1</v>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>The Rising of the Shield Hero</t>
+          <t>Tokyo Ghoul</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -990,14 +1200,19 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Tate no Yuusha no Nariagari</t>
+          <t>Bleach</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bleach</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1006,16 +1221,26 @@
       <c r="D30" t="n">
         <v>1</v>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Re Zero</t>
+          <t>Bleach</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1026,14 +1251,19 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Re Zero kara Hajimeru Isekai Seikatsu</t>
+          <t>Bleach Thousand-Year Blood War</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Bleach Thousand-Year Blood War</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1042,16 +1272,26 @@
       <c r="D32" t="n">
         <v>1</v>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>No Game No Life</t>
+          <t>Bleach Thousand-Year Blood War</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1062,14 +1302,19 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Overlord</t>
+          <t>Hunter x Hunter</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Hunter x Hunter</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1078,16 +1323,26 @@
       <c r="D34" t="n">
         <v>1</v>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mushoku Tensei</t>
+          <t>Hunter x Hunter</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1098,14 +1353,19 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>That Time I Got Reincarnated as a Slime</t>
+          <t>Black Clover</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Black Clover</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1114,16 +1374,26 @@
       <c r="D36" t="n">
         <v>1</v>
       </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Tensei Shitara Slime Datta Ken</t>
+          <t>Black Clover</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1134,14 +1404,19 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Frieren Beyond Journey's End</t>
+          <t>My Hero Academia</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>My Hero Academia</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1150,16 +1425,26 @@
       <c r="D38" t="n">
         <v>1</v>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Sousou no Frieren</t>
+          <t>My Hero Academia</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1170,14 +1455,19 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Made in Abyss</t>
+          <t>Boku no Hero Academia</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Boku no Hero Academia</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1186,16 +1476,26 @@
       <c r="D40" t="n">
         <v>1</v>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Steins Gate</t>
+          <t>Boku no Hero Academia</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1206,14 +1506,19 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Cowboy Bebop</t>
+          <t>Chainsaw Man</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Chainsaw Man</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1222,16 +1527,26 @@
       <c r="D42" t="n">
         <v>1</v>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Neon Genesis Evangelion</t>
+          <t>Chainsaw Man</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1242,14 +1557,19 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Code Geass</t>
+          <t>Solo Leveling</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Solo Leveling</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1258,16 +1578,26 @@
       <c r="D44" t="n">
         <v>1</v>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Akame ga Kill</t>
+          <t>Solo Leveling</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1278,14 +1608,19 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Another</t>
+          <t>Sword Art Online</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Sword Art Online</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1294,16 +1629,26 @@
       <c r="D46" t="n">
         <v>1</v>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Erased</t>
+          <t>Sword Art Online</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1314,14 +1659,19 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Mirai Nikki</t>
+          <t>Fairy Tail</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Fairy Tail</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1330,16 +1680,26 @@
       <c r="D48" t="n">
         <v>1</v>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Elfen Lied</t>
+          <t>Fairy Tail</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1350,14 +1710,19 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Toradora</t>
+          <t>Blue Lock</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Blue Lock</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1366,16 +1731,26 @@
       <c r="D50" t="n">
         <v>1</v>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Your Lie in April</t>
+          <t>Blue Lock</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1386,14 +1761,19 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Clannad</t>
+          <t>Haikyuu</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Haikyuu</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1402,16 +1782,26 @@
       <c r="D52" t="n">
         <v>1</v>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Horimiya</t>
+          <t>Haikyuu</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -1422,14 +1812,19 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Kaguya Sama Love is War</t>
+          <t>Kuroko no Basket</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Kuroko no Basket</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1438,16 +1833,26 @@
       <c r="D54" t="n">
         <v>1</v>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Konosuba</t>
+          <t>Kuroko no Basket</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -1458,14 +1863,19 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>The Eminence in Shadow</t>
+          <t>The Rising of the Shield Hero</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>The Rising of the Shield Hero</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1474,16 +1884,26 @@
       <c r="D56" t="n">
         <v>1</v>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Classroom of the Elite</t>
+          <t>The Rising of the Shield Hero</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1494,14 +1914,19 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DanMachi</t>
+          <t>Tate no Yuusha no Nariagari</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Tate no Yuusha no Nariagari</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1510,16 +1935,26 @@
       <c r="D58" t="n">
         <v>1</v>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Is It Wrong to Try to Pick Up Girls in a Dungeon</t>
+          <t>Tate no Yuusha no Nariagari</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -1530,14 +1965,19 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>High School DxD</t>
+          <t>Re Zero</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Re Zero</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -1546,16 +1986,26 @@
       <c r="D60" t="n">
         <v>1</v>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>To Love Ru</t>
+          <t>Re Zero</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -1566,14 +2016,19 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Date A Live</t>
+          <t>Re Zero kara Hajimeru Isekai Seikatsu</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Re Zero kara Hajimeru Isekai Seikatsu</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -1582,16 +2037,26 @@
       <c r="D62" t="n">
         <v>1</v>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>The Testament of Sister New Devil</t>
+          <t>Re Zero kara Hajimeru Isekai Seikatsu</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -1602,14 +2067,19 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Prison School</t>
+          <t>No Game No Life</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>No Game No Life</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -1618,16 +2088,26 @@
       <c r="D64" t="n">
         <v>1</v>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Redo of Healer</t>
+          <t>No Game No Life</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -1638,14 +2118,19 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Highschool of the Dead</t>
+          <t>Overlord</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Overlord</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -1654,16 +2139,26 @@
       <c r="D66" t="n">
         <v>1</v>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Hellsing Ultimate</t>
+          <t>Overlord</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -1674,14 +2169,19 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Berserk</t>
+          <t>Mushoku Tensei</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Mushoku Tensei</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -1690,16 +2190,26 @@
       <c r="D68" t="n">
         <v>1</v>
       </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Vinland Saga</t>
+          <t>Mushoku Tensei</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -1710,14 +2220,19 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Dororo</t>
+          <t>That Time I Got Reincarnated as a Slime</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>That Time I Got Reincarnated as a Slime</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -1726,16 +2241,26 @@
       <c r="D70" t="n">
         <v>1</v>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Mob Psycho 100</t>
+          <t>That Time I Got Reincarnated as a Slime</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -1746,14 +2271,19 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>One Punch Man</t>
+          <t>Tensei Shitara Slime Datta Ken</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Tensei Shitara Slime Datta Ken</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -1762,16 +2292,26 @@
       <c r="D72" t="n">
         <v>1</v>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Dr Stone</t>
+          <t>Tensei Shitara Slime Datta Ken</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -1782,14 +2322,19 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Fire Force</t>
+          <t>Frieren Beyond Journey's End</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Frieren Beyond Journey's End</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -1798,16 +2343,26 @@
       <c r="D74" t="n">
         <v>1</v>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>The Seven Deadly Sins</t>
+          <t>Frieren Beyond Journey's End</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -1818,14 +2373,19 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Nanatsu no Taizai</t>
+          <t>Sousou no Frieren</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Sousou no Frieren</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -1834,16 +2394,26 @@
       <c r="D76" t="n">
         <v>1</v>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Pokémon</t>
+          <t>Sousou no Frieren</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -1854,14 +2424,19 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Digimon Adventure</t>
+          <t>Made in Abyss</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -1870,16 +2445,26 @@
       <c r="D78" t="n">
         <v>1</v>
       </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Yu Yu Hakusho</t>
+          <t>Made in Abyss</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -1890,14 +2475,19 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Inuyasha</t>
+          <t>Steins Gate</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Steins Gate</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -1906,16 +2496,26 @@
       <c r="D80" t="n">
         <v>1</v>
       </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Provider bloqueou a requisição (403)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Sailor Moon</t>
+          <t>Steins Gate</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -1926,25 +2526,2098 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>Nenhuma variação retornou link válido</t>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
+          <t>Cowboy Bebop</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Cowboy Bebop</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Cowboy Bebop</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" t="n">
+        <v>1</v>
+      </c>
+      <c r="K83" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Neon Genesis Evangelion</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Neon Genesis Evangelion</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>1</v>
+      </c>
+      <c r="D84" t="n">
+        <v>1</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Neon Genesis Evangelion</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" t="n">
+        <v>1</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Code Geass</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Code Geass</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Code Geass</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1</v>
+      </c>
+      <c r="D87" t="n">
+        <v>1</v>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Akame ga Kill</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Akame ga Kill</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" t="n">
+        <v>1</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Akame ga Kill</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" t="n">
+        <v>1</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Another</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Another</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Another</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>1</v>
+      </c>
+      <c r="D91" t="n">
+        <v>1</v>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Erased</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Erased</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>1</v>
+      </c>
+      <c r="D92" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Erased</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1</v>
+      </c>
+      <c r="D93" t="n">
+        <v>1</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Mirai Nikki</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Mirai Nikki</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1</v>
+      </c>
+      <c r="D94" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Mirai Nikki</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" t="n">
+        <v>1</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Elfen Lied</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Elfen Lied</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>1</v>
+      </c>
+      <c r="D96" t="n">
+        <v>1</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Elfen Lied</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>1</v>
+      </c>
+      <c r="D97" t="n">
+        <v>1</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Toradora</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Toradora</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>1</v>
+      </c>
+      <c r="D98" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Toradora</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>1</v>
+      </c>
+      <c r="D99" t="n">
+        <v>1</v>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Your Lie in April</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Your Lie in April</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Your Lie in April</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" t="n">
+        <v>1</v>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Clannad</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Clannad</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Clannad</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>1</v>
+      </c>
+      <c r="D103" t="n">
+        <v>1</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Horimiya</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Horimiya</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>1</v>
+      </c>
+      <c r="D104" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Horimiya</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>1</v>
+      </c>
+      <c r="D105" t="n">
+        <v>1</v>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Kaguya Sama Love is War</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Kaguya Sama Love is War</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Kaguya Sama Love is War</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>1</v>
+      </c>
+      <c r="D107" t="n">
+        <v>1</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Konosuba</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Konosuba</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>1</v>
+      </c>
+      <c r="D108" t="n">
+        <v>1</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Konosuba</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" t="n">
+        <v>1</v>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>The Eminence in Shadow</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>The Eminence in Shadow</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>1</v>
+      </c>
+      <c r="D110" t="n">
+        <v>1</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>The Eminence in Shadow</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>1</v>
+      </c>
+      <c r="D111" t="n">
+        <v>1</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Classroom of the Elite</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Classroom of the Elite</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Classroom of the Elite</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" t="n">
+        <v>1</v>
+      </c>
+      <c r="K113" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>DanMachi</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>DanMachi</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" t="n">
+        <v>1</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>DanMachi</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>1</v>
+      </c>
+      <c r="D115" t="n">
+        <v>1</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Is It Wrong to Try to Pick Up Girls in a Dungeon</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Is It Wrong to Try to Pick Up Girls in a Dungeon</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>1</v>
+      </c>
+      <c r="D116" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Is It Wrong to Try to Pick Up Girls in a Dungeon</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>1</v>
+      </c>
+      <c r="D117" t="n">
+        <v>1</v>
+      </c>
+      <c r="K117" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>High School DxD</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>High School DxD</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>1</v>
+      </c>
+      <c r="D118" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>High School DxD</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>1</v>
+      </c>
+      <c r="D119" t="n">
+        <v>1</v>
+      </c>
+      <c r="K119" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>To Love Ru</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>To Love Ru</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>To Love Ru</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>1</v>
+      </c>
+      <c r="D121" t="n">
+        <v>1</v>
+      </c>
+      <c r="K121" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Date A Live</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Date A Live</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" t="n">
+        <v>1</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Date A Live</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>1</v>
+      </c>
+      <c r="D123" t="n">
+        <v>1</v>
+      </c>
+      <c r="K123" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>The Testament of Sister New Devil</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>The Testament of Sister New Devil</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>1</v>
+      </c>
+      <c r="D124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>The Testament of Sister New Devil</t>
+        </is>
+      </c>
+      <c r="C125" t="n">
+        <v>1</v>
+      </c>
+      <c r="D125" t="n">
+        <v>1</v>
+      </c>
+      <c r="K125" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Prison School</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Prison School</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>1</v>
+      </c>
+      <c r="D126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Prison School</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>1</v>
+      </c>
+      <c r="D127" t="n">
+        <v>1</v>
+      </c>
+      <c r="K127" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Redo of Healer</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Redo of Healer</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" t="n">
+        <v>1</v>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Redo of Healer</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>1</v>
+      </c>
+      <c r="D129" t="n">
+        <v>1</v>
+      </c>
+      <c r="K129" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Highschool of the Dead</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Highschool of the Dead</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>1</v>
+      </c>
+      <c r="D130" t="n">
+        <v>1</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Highschool of the Dead</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>1</v>
+      </c>
+      <c r="D131" t="n">
+        <v>1</v>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Hellsing Ultimate</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Hellsing Ultimate</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>1</v>
+      </c>
+      <c r="D132" t="n">
+        <v>1</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Hellsing Ultimate</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>1</v>
+      </c>
+      <c r="D133" t="n">
+        <v>1</v>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Berserk</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Berserk</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>1</v>
+      </c>
+      <c r="D134" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Berserk</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" t="n">
+        <v>1</v>
+      </c>
+      <c r="K135" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Vinland Saga</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Vinland Saga</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>1</v>
+      </c>
+      <c r="D136" t="n">
+        <v>1</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Vinland Saga</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" t="n">
+        <v>1</v>
+      </c>
+      <c r="K137" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Dororo</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Dororo</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>1</v>
+      </c>
+      <c r="D138" t="n">
+        <v>1</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Dororo</t>
+        </is>
+      </c>
+      <c r="C139" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" t="n">
+        <v>1</v>
+      </c>
+      <c r="K139" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Mob Psycho 100</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Mob Psycho 100</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>1</v>
+      </c>
+      <c r="D140" t="n">
+        <v>1</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K140" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Mob Psycho 100</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>1</v>
+      </c>
+      <c r="D141" t="n">
+        <v>1</v>
+      </c>
+      <c r="K141" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>One Punch Man</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>One Punch Man</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>1</v>
+      </c>
+      <c r="D142" t="n">
+        <v>1</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>One Punch Man</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>1</v>
+      </c>
+      <c r="D143" t="n">
+        <v>1</v>
+      </c>
+      <c r="K143" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Dr Stone</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Dr Stone</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>1</v>
+      </c>
+      <c r="D144" t="n">
+        <v>1</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Dr Stone</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>1</v>
+      </c>
+      <c r="D145" t="n">
+        <v>1</v>
+      </c>
+      <c r="K145" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Fire Force</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Fire Force</t>
+        </is>
+      </c>
+      <c r="C146" t="n">
+        <v>1</v>
+      </c>
+      <c r="D146" t="n">
+        <v>1</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Fire Force</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>1</v>
+      </c>
+      <c r="D147" t="n">
+        <v>1</v>
+      </c>
+      <c r="K147" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>The Seven Deadly Sins</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>The Seven Deadly Sins</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>1</v>
+      </c>
+      <c r="D148" t="n">
+        <v>1</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>The Seven Deadly Sins</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>1</v>
+      </c>
+      <c r="D149" t="n">
+        <v>1</v>
+      </c>
+      <c r="K149" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Nanatsu no Taizai</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Nanatsu no Taizai</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>1</v>
+      </c>
+      <c r="D150" t="n">
+        <v>1</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K150" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Nanatsu no Taizai</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>1</v>
+      </c>
+      <c r="D151" t="n">
+        <v>1</v>
+      </c>
+      <c r="K151" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Pokémon</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Pokémon</t>
+        </is>
+      </c>
+      <c r="C152" t="n">
+        <v>1</v>
+      </c>
+      <c r="D152" t="n">
+        <v>1</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K152" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Pokémon</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" t="n">
+        <v>1</v>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Digimon Adventure</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Digimon Adventure</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>1</v>
+      </c>
+      <c r="D154" t="n">
+        <v>1</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Digimon Adventure</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" t="n">
+        <v>1</v>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Yu Yu Hakusho</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Yu Yu Hakusho</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>1</v>
+      </c>
+      <c r="D156" t="n">
+        <v>1</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Yu Yu Hakusho</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" t="n">
+        <v>1</v>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Inuyasha</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Inuyasha</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" t="n">
+        <v>1</v>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Inuyasha</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>1</v>
+      </c>
+      <c r="D159" t="n">
+        <v>1</v>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Sailor Moon</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Sailor Moon</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="n">
+        <v>1</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Sailor Moon</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>1</v>
+      </c>
+      <c r="D161" t="n">
+        <v>1</v>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
           <t>Cardcaptor Sakura</t>
         </is>
       </c>
-      <c r="C82" t="n">
-        <v>1</v>
-      </c>
-      <c r="D82" t="n">
-        <v>1</v>
-      </c>
-      <c r="K82" t="inlineStr">
-        <is>
-          <t>Nenhuma variação retornou link válido</t>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Cardcaptor Sakura</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>1</v>
+      </c>
+      <c r="D162" t="n">
+        <v>1</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>provider_interno_1</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>provider-interno-1</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>Provider bloqueou a requisição (403)</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Cardcaptor Sakura</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>1</v>
+      </c>
+      <c r="D163" t="n">
+        <v>1</v>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>Nenhum provider retornou link válido</t>
         </is>
       </c>
     </row>

</xml_diff>